<commit_message>
Changed Daily and Weekly graph
</commit_message>
<xml_diff>
--- a/Optimisation/Output/Main_results.xlsx
+++ b/Optimisation/Output/Main_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT28"/>
+  <dimension ref="A1:AU44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -657,6 +657,11 @@
       <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>DA_Price_Forecast</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>Dispatch_Model</t>
         </is>
       </c>
     </row>
@@ -815,6 +820,7 @@
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="inlineStr"/>
       <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -979,6 +985,7 @@
         <v>-140838.28</v>
       </c>
       <c r="AT3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1143,6 +1150,7 @@
         <v>-216061.57</v>
       </c>
       <c r="AT4" t="inlineStr"/>
+      <c r="AU4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1307,6 +1315,7 @@
         <v>-116643.32</v>
       </c>
       <c r="AT5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1471,6 +1480,7 @@
         <v>-209191.16</v>
       </c>
       <c r="AT6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1635,6 +1645,7 @@
         <v>-163612.59</v>
       </c>
       <c r="AT7" t="inlineStr"/>
+      <c r="AU7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1799,6 +1810,7 @@
         <v>-146414.61</v>
       </c>
       <c r="AT8" t="inlineStr"/>
+      <c r="AU8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1963,6 +1975,7 @@
         <v>-122141.9</v>
       </c>
       <c r="AT9" t="inlineStr"/>
+      <c r="AU9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2127,6 +2140,7 @@
         <v>-113682.66</v>
       </c>
       <c r="AT10" t="inlineStr"/>
+      <c r="AU10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2291,6 +2305,7 @@
         <v>-193860.34</v>
       </c>
       <c r="AT11" t="inlineStr"/>
+      <c r="AU11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2455,6 +2470,7 @@
         <v>-217395.65</v>
       </c>
       <c r="AT12" t="inlineStr"/>
+      <c r="AU12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2619,6 +2635,7 @@
         <v>-239812.86</v>
       </c>
       <c r="AT13" t="inlineStr"/>
+      <c r="AU13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2783,6 +2800,7 @@
         <v>-258223.11</v>
       </c>
       <c r="AT14" t="inlineStr"/>
+      <c r="AU14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2947,6 +2965,7 @@
         <v>-140838.28</v>
       </c>
       <c r="AT15" t="inlineStr"/>
+      <c r="AU15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3111,6 +3130,7 @@
         <v>-108524.42</v>
       </c>
       <c r="AT16" t="inlineStr"/>
+      <c r="AU16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3275,6 +3295,7 @@
         <v>-170105.4</v>
       </c>
       <c r="AT17" t="inlineStr"/>
+      <c r="AU17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3439,6 +3460,7 @@
         <v>-237524.78</v>
       </c>
       <c r="AT18" t="inlineStr"/>
+      <c r="AU18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3603,6 +3625,7 @@
         <v>-331310.59</v>
       </c>
       <c r="AT19" t="inlineStr"/>
+      <c r="AU19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3767,6 +3790,7 @@
         <v>-353133.75</v>
       </c>
       <c r="AT20" t="inlineStr"/>
+      <c r="AU20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3931,6 +3955,7 @@
         <v>-257965.55</v>
       </c>
       <c r="AT21" t="inlineStr"/>
+      <c r="AU21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4095,6 +4120,7 @@
         <v>-170532.18</v>
       </c>
       <c r="AT22" t="inlineStr"/>
+      <c r="AU22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4259,6 +4285,7 @@
         <v>-116643.32</v>
       </c>
       <c r="AT23" t="inlineStr"/>
+      <c r="AU23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4423,6 +4450,7 @@
         <v>0</v>
       </c>
       <c r="AT24" t="inlineStr"/>
+      <c r="AU24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4591,6 +4619,7 @@
           <t>MAPE_05</t>
         </is>
       </c>
+      <c r="AU25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4759,6 +4788,7 @@
           <t>MAPE_05</t>
         </is>
       </c>
+      <c r="AU26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4927,6 +4957,7 @@
           <t>MAPE_15</t>
         </is>
       </c>
+      <c r="AU27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5093,6 +5124,2539 @@
       <c r="AT28" t="inlineStr">
         <is>
           <t>MAPE_15</t>
+        </is>
+      </c>
+      <c r="AU28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-05-15 11:20</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ROLLING_MEAN</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>SEASONAL_PREDICTION</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="F29" t="b">
+        <v>1</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>HYDRO_COUPLED</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>500</v>
+      </c>
+      <c r="I29" t="n">
+        <v>1</v>
+      </c>
+      <c r="J29" t="n">
+        <v>80</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L29" t="n">
+        <v>15</v>
+      </c>
+      <c r="M29" t="n">
+        <v>5</v>
+      </c>
+      <c r="N29" t="n">
+        <v>8</v>
+      </c>
+      <c r="O29" t="n">
+        <v>4000</v>
+      </c>
+      <c r="P29" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>-269837.73</v>
+      </c>
+      <c r="R29" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="S29" t="n">
+        <v>-142777.3</v>
+      </c>
+      <c r="T29" t="n">
+        <v>127060.43</v>
+      </c>
+      <c r="U29" t="n">
+        <v>298</v>
+      </c>
+      <c r="V29" t="n">
+        <v>68</v>
+      </c>
+      <c r="W29" t="n">
+        <v>17145.2</v>
+      </c>
+      <c r="X29" t="n">
+        <v>499.1</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>143.1</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>3487.09</v>
+      </c>
+      <c r="AA29" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="AB29" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="AC29" t="n">
+        <v>366</v>
+      </c>
+      <c r="AD29" t="n">
+        <v>3477.57</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>150000</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>-155366</v>
+      </c>
+      <c r="AG29" t="inlineStr">
+        <is>
+          <t>&gt;100</t>
+        </is>
+      </c>
+      <c r="AH29" t="n">
+        <v>0.6820000000000001</v>
+      </c>
+      <c r="AI29" t="n">
+        <v>97.8</v>
+      </c>
+      <c r="AJ29" t="n">
+        <v>199424.99</v>
+      </c>
+      <c r="AK29" t="n">
+        <v>145228.09</v>
+      </c>
+      <c r="AL29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM29" t="n">
+        <v>-382659.74</v>
+      </c>
+      <c r="AN29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO29" t="inlineStr">
+        <is>
+          <t>RBD_ID_500kWh_FCROLLING_MEAN_PFSP_LFCNN_LSTM_DAM05.xlsx</t>
+        </is>
+      </c>
+      <c r="AP29" t="n">
+        <v>-80560.36</v>
+      </c>
+      <c r="AQ29" t="n">
+        <v>-189277.37</v>
+      </c>
+      <c r="AR29" t="n">
+        <v>-6038.01</v>
+      </c>
+      <c r="AS29" t="n">
+        <v>-136739.29</v>
+      </c>
+      <c r="AT29" t="inlineStr">
+        <is>
+          <t>MAPE_05</t>
+        </is>
+      </c>
+      <c r="AU29" t="inlineStr">
+        <is>
+          <t>RULE_BASED_DISPATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-05-15 12:25</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ROLLING_MEAN</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SEASONAL_PREDICTION</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="F30" t="b">
+        <v>1</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>DAY_AHEAD</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>500</v>
+      </c>
+      <c r="I30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J30" t="n">
+        <v>80</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L30" t="n">
+        <v>15</v>
+      </c>
+      <c r="M30" t="n">
+        <v>5</v>
+      </c>
+      <c r="N30" t="n">
+        <v>8</v>
+      </c>
+      <c r="O30" t="n">
+        <v>4000</v>
+      </c>
+      <c r="P30" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>-269837.73</v>
+      </c>
+      <c r="R30" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="S30" t="n">
+        <v>-150080.62</v>
+      </c>
+      <c r="T30" t="n">
+        <v>119757.11</v>
+      </c>
+      <c r="U30" t="n">
+        <v>291</v>
+      </c>
+      <c r="V30" t="n">
+        <v>75</v>
+      </c>
+      <c r="W30" t="n">
+        <v>17123.6</v>
+      </c>
+      <c r="X30" t="n">
+        <v>531.3</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>143.7</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>9391.98</v>
+      </c>
+      <c r="AA30" t="n">
+        <v>465.1</v>
+      </c>
+      <c r="AB30" t="n">
+        <v>463.8</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>366</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>-7603.21</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>150000</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>-250616</v>
+      </c>
+      <c r="AG30" t="inlineStr">
+        <is>
+          <t>&gt;100</t>
+        </is>
+      </c>
+      <c r="AH30" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="AI30" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="AJ30" t="n">
+        <v>222256.8</v>
+      </c>
+      <c r="AK30" t="n">
+        <v>145228.09</v>
+      </c>
+      <c r="AL30" t="n">
+        <v>-17016.02</v>
+      </c>
+      <c r="AM30" t="n">
+        <v>-406889.98</v>
+      </c>
+      <c r="AN30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO30" t="inlineStr">
+        <is>
+          <t>RBD_DA_500kWh_FCROLLING_MEAN_PFSP_LFCNN_LSTM_DAM05.xlsx</t>
+        </is>
+      </c>
+      <c r="AP30" t="n">
+        <v>-80560.36</v>
+      </c>
+      <c r="AQ30" t="n">
+        <v>-189277.37</v>
+      </c>
+      <c r="AR30" t="n">
+        <v>-5938.37</v>
+      </c>
+      <c r="AS30" t="n">
+        <v>-144142.24</v>
+      </c>
+      <c r="AT30" t="inlineStr">
+        <is>
+          <t>MAPE_05</t>
+        </is>
+      </c>
+      <c r="AU30" t="inlineStr">
+        <is>
+          <t>RULE_BASED_DISPATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-05-15 12:56</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ROLLING_MEAN</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>SEASONAL_PREDICTION</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="F31" t="b">
+        <v>1</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>HYDRO_COUPLED</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>6000</v>
+      </c>
+      <c r="I31" t="n">
+        <v>1</v>
+      </c>
+      <c r="J31" t="n">
+        <v>80</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L31" t="n">
+        <v>15</v>
+      </c>
+      <c r="M31" t="n">
+        <v>5</v>
+      </c>
+      <c r="N31" t="n">
+        <v>8</v>
+      </c>
+      <c r="O31" t="n">
+        <v>48000</v>
+      </c>
+      <c r="P31" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>-269837.73</v>
+      </c>
+      <c r="R31" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="S31" t="n">
+        <v>-141675.73</v>
+      </c>
+      <c r="T31" t="n">
+        <v>128162</v>
+      </c>
+      <c r="U31" t="n">
+        <v>292</v>
+      </c>
+      <c r="V31" t="n">
+        <v>74</v>
+      </c>
+      <c r="W31" t="n">
+        <v>17220</v>
+      </c>
+      <c r="X31" t="n">
+        <v>377.9</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>147</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>12218.19</v>
+      </c>
+      <c r="AA31" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="AB31" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>366</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>-60418.72</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>-2916665</v>
+      </c>
+      <c r="AG31" t="inlineStr">
+        <is>
+          <t>&gt;100</t>
+        </is>
+      </c>
+      <c r="AH31" t="n">
+        <v>0.928</v>
+      </c>
+      <c r="AI31" t="n">
+        <v>98.40000000000001</v>
+      </c>
+      <c r="AJ31" t="n">
+        <v>285825.37</v>
+      </c>
+      <c r="AK31" t="n">
+        <v>145228.09</v>
+      </c>
+      <c r="AL31" t="n">
+        <v>-72802.44</v>
+      </c>
+      <c r="AM31" t="n">
+        <v>-459227.44</v>
+      </c>
+      <c r="AN31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO31" t="inlineStr">
+        <is>
+          <t>RBD_ID_6000kWh_FCROLLING_MEAN_PFSP_LFCNN_LSTM_DAM05.xlsx</t>
+        </is>
+      </c>
+      <c r="AP31" t="n">
+        <v>-80560.36</v>
+      </c>
+      <c r="AQ31" t="n">
+        <v>-189277.37</v>
+      </c>
+      <c r="AR31" t="n">
+        <v>-6504.54</v>
+      </c>
+      <c r="AS31" t="n">
+        <v>-135171.19</v>
+      </c>
+      <c r="AT31" t="inlineStr">
+        <is>
+          <t>MAPE_05</t>
+        </is>
+      </c>
+      <c r="AU31" t="inlineStr">
+        <is>
+          <t>RULE_BASED_DISPATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-05-15 13:45</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ROLLING_MEAN</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>SEASONAL_PREDICTION</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="F32" t="b">
+        <v>1</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>HYDRO_COUPLED</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J32" t="n">
+        <v>80</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L32" t="n">
+        <v>15</v>
+      </c>
+      <c r="M32" t="n">
+        <v>5</v>
+      </c>
+      <c r="N32" t="n">
+        <v>8</v>
+      </c>
+      <c r="O32" t="n">
+        <v>24000</v>
+      </c>
+      <c r="P32" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>-269837.73</v>
+      </c>
+      <c r="R32" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="S32" t="n">
+        <v>-142519.49</v>
+      </c>
+      <c r="T32" t="n">
+        <v>127318.24</v>
+      </c>
+      <c r="U32" t="n">
+        <v>298</v>
+      </c>
+      <c r="V32" t="n">
+        <v>68</v>
+      </c>
+      <c r="W32" t="n">
+        <v>17188.4</v>
+      </c>
+      <c r="X32" t="n">
+        <v>431.9</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>144.9</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>9738.51</v>
+      </c>
+      <c r="AA32" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="AB32" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="AC32" t="n">
+        <v>366</v>
+      </c>
+      <c r="AD32" t="n">
+        <v>-1730.88</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>900000</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>-1164511</v>
+      </c>
+      <c r="AG32" t="inlineStr">
+        <is>
+          <t>&gt;100</t>
+        </is>
+      </c>
+      <c r="AH32" t="n">
+        <v>0.747</v>
+      </c>
+      <c r="AI32" t="n">
+        <v>98</v>
+      </c>
+      <c r="AJ32" t="n">
+        <v>224867.54</v>
+      </c>
+      <c r="AK32" t="n">
+        <v>145228.09</v>
+      </c>
+      <c r="AL32" t="n">
+        <v>-11474.13</v>
+      </c>
+      <c r="AM32" t="n">
+        <v>-401593.07</v>
+      </c>
+      <c r="AN32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO32" t="inlineStr">
+        <is>
+          <t>RBD_ID_3000kWh_FCROLLING_MEAN_PFSP_LFCNN_LSTM_DAM05.xlsx</t>
+        </is>
+      </c>
+      <c r="AP32" t="n">
+        <v>-80560.36</v>
+      </c>
+      <c r="AQ32" t="n">
+        <v>-189277.37</v>
+      </c>
+      <c r="AR32" t="n">
+        <v>-6298</v>
+      </c>
+      <c r="AS32" t="n">
+        <v>-136221.49</v>
+      </c>
+      <c r="AT32" t="inlineStr">
+        <is>
+          <t>MAPE_05</t>
+        </is>
+      </c>
+      <c r="AU32" t="inlineStr">
+        <is>
+          <t>RULE_BASED_DISPATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:03</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ROLLING_MEAN</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>SEASONAL_PREDICTION</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="F33" t="b">
+        <v>1</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>HYDRO_COUPLED</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I33" t="n">
+        <v>1</v>
+      </c>
+      <c r="J33" t="n">
+        <v>80</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L33" t="n">
+        <v>15</v>
+      </c>
+      <c r="M33" t="n">
+        <v>5</v>
+      </c>
+      <c r="N33" t="n">
+        <v>8</v>
+      </c>
+      <c r="O33" t="n">
+        <v>8000</v>
+      </c>
+      <c r="P33" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>-269837.73</v>
+      </c>
+      <c r="R33" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="S33" t="n">
+        <v>-142571.18</v>
+      </c>
+      <c r="T33" t="n">
+        <v>127266.55</v>
+      </c>
+      <c r="U33" t="n">
+        <v>303</v>
+      </c>
+      <c r="V33" t="n">
+        <v>63</v>
+      </c>
+      <c r="W33" t="n">
+        <v>17155.3</v>
+      </c>
+      <c r="X33" t="n">
+        <v>484.6</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>143.6</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>5666.41</v>
+      </c>
+      <c r="AA33" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="AB33" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>366</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>6321.09</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>300000</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>-317237</v>
+      </c>
+      <c r="AG33" t="inlineStr">
+        <is>
+          <t>&gt;100</t>
+        </is>
+      </c>
+      <c r="AH33" t="n">
+        <v>0.661</v>
+      </c>
+      <c r="AI33" t="n">
+        <v>97.7</v>
+      </c>
+      <c r="AJ33" t="n">
+        <v>199064.75</v>
+      </c>
+      <c r="AK33" t="n">
+        <v>145228.09</v>
+      </c>
+      <c r="AL33" t="n">
+        <v>672</v>
+      </c>
+      <c r="AM33" t="n">
+        <v>-379914.06</v>
+      </c>
+      <c r="AN33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO33" t="inlineStr">
+        <is>
+          <t>RBD_ID_1000kWh_FCROLLING_MEAN_PFSP_LFCNN_LSTM_DAM05.xlsx</t>
+        </is>
+      </c>
+      <c r="AP33" t="n">
+        <v>-80560.36</v>
+      </c>
+      <c r="AQ33" t="n">
+        <v>-189277.37</v>
+      </c>
+      <c r="AR33" t="n">
+        <v>-6162.14</v>
+      </c>
+      <c r="AS33" t="n">
+        <v>-136409.04</v>
+      </c>
+      <c r="AT33" t="inlineStr">
+        <is>
+          <t>MAPE_05</t>
+        </is>
+      </c>
+      <c r="AU33" t="inlineStr">
+        <is>
+          <t>RULE_BASED_DISPATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:08</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ROLLING_MEAN</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>SEASONAL_PREDICTION</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="F34" t="b">
+        <v>1</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>HYDRO_COUPLED</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I34" t="n">
+        <v>1</v>
+      </c>
+      <c r="J34" t="n">
+        <v>80</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L34" t="n">
+        <v>15</v>
+      </c>
+      <c r="M34" t="n">
+        <v>5</v>
+      </c>
+      <c r="N34" t="n">
+        <v>8</v>
+      </c>
+      <c r="O34" t="n">
+        <v>24000</v>
+      </c>
+      <c r="P34" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>-269837.73</v>
+      </c>
+      <c r="R34" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="S34" t="n">
+        <v>-142519.49</v>
+      </c>
+      <c r="T34" t="n">
+        <v>127318.24</v>
+      </c>
+      <c r="U34" t="n">
+        <v>298</v>
+      </c>
+      <c r="V34" t="n">
+        <v>68</v>
+      </c>
+      <c r="W34" t="n">
+        <v>17188.4</v>
+      </c>
+      <c r="X34" t="n">
+        <v>431.9</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>144.9</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>9738.51</v>
+      </c>
+      <c r="AA34" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="AB34" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="AC34" t="n">
+        <v>366</v>
+      </c>
+      <c r="AD34" t="n">
+        <v>-1730.88</v>
+      </c>
+      <c r="AE34" t="n">
+        <v>900000</v>
+      </c>
+      <c r="AF34" t="n">
+        <v>-1164511</v>
+      </c>
+      <c r="AG34" t="inlineStr">
+        <is>
+          <t>&gt;100</t>
+        </is>
+      </c>
+      <c r="AH34" t="n">
+        <v>0.747</v>
+      </c>
+      <c r="AI34" t="n">
+        <v>98</v>
+      </c>
+      <c r="AJ34" t="n">
+        <v>224867.54</v>
+      </c>
+      <c r="AK34" t="n">
+        <v>145228.09</v>
+      </c>
+      <c r="AL34" t="n">
+        <v>-11474.13</v>
+      </c>
+      <c r="AM34" t="n">
+        <v>-401593.07</v>
+      </c>
+      <c r="AN34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO34" t="inlineStr">
+        <is>
+          <t>RBD_ID_3000kWh_FCROLLING_MEAN_PFSP_LFCNN_LSTM_DAM05.xlsx</t>
+        </is>
+      </c>
+      <c r="AP34" t="n">
+        <v>-80560.36</v>
+      </c>
+      <c r="AQ34" t="n">
+        <v>-189277.37</v>
+      </c>
+      <c r="AR34" t="n">
+        <v>-6298</v>
+      </c>
+      <c r="AS34" t="n">
+        <v>-136221.49</v>
+      </c>
+      <c r="AT34" t="inlineStr">
+        <is>
+          <t>MAPE_05</t>
+        </is>
+      </c>
+      <c r="AU34" t="inlineStr">
+        <is>
+          <t>RULE_BASED_DISPATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:11</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ROLLING_MEAN</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>SEASONAL_PREDICTION</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="F35" t="b">
+        <v>1</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>HYDRO_COUPLED</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>200</v>
+      </c>
+      <c r="I35" t="n">
+        <v>1</v>
+      </c>
+      <c r="J35" t="n">
+        <v>80</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L35" t="n">
+        <v>15</v>
+      </c>
+      <c r="M35" t="n">
+        <v>5</v>
+      </c>
+      <c r="N35" t="n">
+        <v>8</v>
+      </c>
+      <c r="O35" t="n">
+        <v>1600</v>
+      </c>
+      <c r="P35" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>-269837.73</v>
+      </c>
+      <c r="R35" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="S35" t="n">
+        <v>-144627.7</v>
+      </c>
+      <c r="T35" t="n">
+        <v>125210.03</v>
+      </c>
+      <c r="U35" t="n">
+        <v>293</v>
+      </c>
+      <c r="V35" t="n">
+        <v>73</v>
+      </c>
+      <c r="W35" t="n">
+        <v>17136.7</v>
+      </c>
+      <c r="X35" t="n">
+        <v>513.4</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>142.6</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>1212.6</v>
+      </c>
+      <c r="AA35" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="AB35" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="AC35" t="n">
+        <v>366</v>
+      </c>
+      <c r="AD35" t="n">
+        <v>1209.29</v>
+      </c>
+      <c r="AE35" t="n">
+        <v>60000</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>-64015</v>
+      </c>
+      <c r="AG35" t="inlineStr">
+        <is>
+          <t>&gt;100</t>
+        </is>
+      </c>
+      <c r="AH35" t="n">
+        <v>0.727</v>
+      </c>
+      <c r="AI35" t="n">
+        <v>97.90000000000001</v>
+      </c>
+      <c r="AJ35" t="n">
+        <v>207142.81</v>
+      </c>
+      <c r="AK35" t="n">
+        <v>145228.09</v>
+      </c>
+      <c r="AL35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM35" t="n">
+        <v>-394502.46</v>
+      </c>
+      <c r="AN35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO35" t="inlineStr">
+        <is>
+          <t>RBD_ID_200kWh_FCROLLING_MEAN_PFSP_LFCNN_LSTM_DAM05.xlsx</t>
+        </is>
+      </c>
+      <c r="AP35" t="n">
+        <v>-80560.36</v>
+      </c>
+      <c r="AQ35" t="n">
+        <v>-189277.37</v>
+      </c>
+      <c r="AR35" t="n">
+        <v>-5977.29</v>
+      </c>
+      <c r="AS35" t="n">
+        <v>-138650.41</v>
+      </c>
+      <c r="AT35" t="inlineStr">
+        <is>
+          <t>MAPE_05</t>
+        </is>
+      </c>
+      <c r="AU35" t="inlineStr">
+        <is>
+          <t>RULE_BASED_DISPATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:16</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ROLLING_MEAN</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>SEASONAL_PREDICTION</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="F36" t="b">
+        <v>1</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>HYDRO_COUPLED</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>500</v>
+      </c>
+      <c r="I36" t="n">
+        <v>1</v>
+      </c>
+      <c r="J36" t="n">
+        <v>80</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L36" t="n">
+        <v>15</v>
+      </c>
+      <c r="M36" t="n">
+        <v>5</v>
+      </c>
+      <c r="N36" t="n">
+        <v>8</v>
+      </c>
+      <c r="O36" t="n">
+        <v>4000</v>
+      </c>
+      <c r="P36" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>-269837.73</v>
+      </c>
+      <c r="R36" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="S36" t="n">
+        <v>-142777.3</v>
+      </c>
+      <c r="T36" t="n">
+        <v>127060.43</v>
+      </c>
+      <c r="U36" t="n">
+        <v>298</v>
+      </c>
+      <c r="V36" t="n">
+        <v>68</v>
+      </c>
+      <c r="W36" t="n">
+        <v>17145.2</v>
+      </c>
+      <c r="X36" t="n">
+        <v>499.1</v>
+      </c>
+      <c r="Y36" t="n">
+        <v>143.1</v>
+      </c>
+      <c r="Z36" t="n">
+        <v>3487.09</v>
+      </c>
+      <c r="AA36" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="AB36" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="AC36" t="n">
+        <v>366</v>
+      </c>
+      <c r="AD36" t="n">
+        <v>3477.57</v>
+      </c>
+      <c r="AE36" t="n">
+        <v>150000</v>
+      </c>
+      <c r="AF36" t="n">
+        <v>-155366</v>
+      </c>
+      <c r="AG36" t="inlineStr">
+        <is>
+          <t>&gt;100</t>
+        </is>
+      </c>
+      <c r="AH36" t="n">
+        <v>0.6820000000000001</v>
+      </c>
+      <c r="AI36" t="n">
+        <v>97.8</v>
+      </c>
+      <c r="AJ36" t="n">
+        <v>199424.99</v>
+      </c>
+      <c r="AK36" t="n">
+        <v>145228.09</v>
+      </c>
+      <c r="AL36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM36" t="n">
+        <v>-382659.74</v>
+      </c>
+      <c r="AN36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO36" t="inlineStr">
+        <is>
+          <t>RBD_ID_500kWh_FCROLLING_MEAN_PFSP_LFCNN_LSTM_DAM05.xlsx</t>
+        </is>
+      </c>
+      <c r="AP36" t="n">
+        <v>-80560.36</v>
+      </c>
+      <c r="AQ36" t="n">
+        <v>-189277.37</v>
+      </c>
+      <c r="AR36" t="n">
+        <v>-6038.01</v>
+      </c>
+      <c r="AS36" t="n">
+        <v>-136739.29</v>
+      </c>
+      <c r="AT36" t="inlineStr">
+        <is>
+          <t>MAPE_05</t>
+        </is>
+      </c>
+      <c r="AU36" t="inlineStr">
+        <is>
+          <t>RULE_BASED_DISPATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:27</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ROLLING_MEAN</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>LP_OPTIMISED</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="F37" t="b">
+        <v>1</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>HYDRO_COUPLED</t>
+        </is>
+      </c>
+      <c r="H37" t="n">
+        <v>500</v>
+      </c>
+      <c r="I37" t="n">
+        <v>1</v>
+      </c>
+      <c r="J37" t="n">
+        <v>80</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L37" t="n">
+        <v>15</v>
+      </c>
+      <c r="M37" t="n">
+        <v>5</v>
+      </c>
+      <c r="N37" t="n">
+        <v>8</v>
+      </c>
+      <c r="O37" t="n">
+        <v>4000</v>
+      </c>
+      <c r="P37" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>-269837.73</v>
+      </c>
+      <c r="R37" t="n">
+        <v>6826.28</v>
+      </c>
+      <c r="S37" t="n">
+        <v>-167988.4</v>
+      </c>
+      <c r="T37" t="n">
+        <v>152620.15</v>
+      </c>
+      <c r="U37" t="n">
+        <v>302</v>
+      </c>
+      <c r="V37" t="n">
+        <v>64</v>
+      </c>
+      <c r="W37" t="n">
+        <v>17190.1</v>
+      </c>
+      <c r="X37" t="n">
+        <v>399.5</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="Z37" t="n">
+        <v>1148.88</v>
+      </c>
+      <c r="AA37" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="AB37" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="AC37" t="n">
+        <v>366</v>
+      </c>
+      <c r="AD37" t="n">
+        <v>34872.59</v>
+      </c>
+      <c r="AE37" t="n">
+        <v>150000</v>
+      </c>
+      <c r="AF37" t="n">
+        <v>166572</v>
+      </c>
+      <c r="AG37" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="AH37" t="n">
+        <v>0.595</v>
+      </c>
+      <c r="AI37" t="n">
+        <v>97.40000000000001</v>
+      </c>
+      <c r="AJ37" t="n">
+        <v>75438.62</v>
+      </c>
+      <c r="AK37" t="n">
+        <v>145228.09</v>
+      </c>
+      <c r="AL37" t="n">
+        <v>33819.25</v>
+      </c>
+      <c r="AM37" t="n">
+        <v>-235451.86</v>
+      </c>
+      <c r="AN37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO37" t="inlineStr">
+        <is>
+          <t>OD_ID_500kWh_FCROLLING_MEAN_PFLP_LFCNN_LSTM_DAM05.xlsx</t>
+        </is>
+      </c>
+      <c r="AP37" t="n">
+        <v>-80560.36</v>
+      </c>
+      <c r="AQ37" t="n">
+        <v>-189277.37</v>
+      </c>
+      <c r="AR37" t="n">
+        <v>-49474.39</v>
+      </c>
+      <c r="AS37" t="n">
+        <v>-118514.01</v>
+      </c>
+      <c r="AT37" t="inlineStr">
+        <is>
+          <t>MAPE_05</t>
+        </is>
+      </c>
+      <c r="AU37" t="inlineStr">
+        <is>
+          <t>OPTIMISATION_DISPATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-05-15 15:16</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ROLLING_MEAN</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>LP_OPTIMISED</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="F38" t="b">
+        <v>1</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>DAY_AHEAD</t>
+        </is>
+      </c>
+      <c r="H38" t="n">
+        <v>500</v>
+      </c>
+      <c r="I38" t="n">
+        <v>1</v>
+      </c>
+      <c r="J38" t="n">
+        <v>80</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L38" t="n">
+        <v>15</v>
+      </c>
+      <c r="M38" t="n">
+        <v>5</v>
+      </c>
+      <c r="N38" t="n">
+        <v>8</v>
+      </c>
+      <c r="O38" t="n">
+        <v>4000</v>
+      </c>
+      <c r="P38" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>-269837.73</v>
+      </c>
+      <c r="R38" t="n">
+        <v>30830.76</v>
+      </c>
+      <c r="S38" t="n">
+        <v>-169632.77</v>
+      </c>
+      <c r="T38" t="n">
+        <v>174980.26</v>
+      </c>
+      <c r="U38" t="n">
+        <v>328</v>
+      </c>
+      <c r="V38" t="n">
+        <v>38</v>
+      </c>
+      <c r="W38" t="n">
+        <v>17048.3</v>
+      </c>
+      <c r="X38" t="n">
+        <v>645.3</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="Z38" t="n">
+        <v>9391.85</v>
+      </c>
+      <c r="AA38" t="n">
+        <v>465</v>
+      </c>
+      <c r="AB38" t="n">
+        <v>463.7</v>
+      </c>
+      <c r="AC38" t="n">
+        <v>366</v>
+      </c>
+      <c r="AD38" t="n">
+        <v>-26898.89</v>
+      </c>
+      <c r="AE38" t="n">
+        <v>150000</v>
+      </c>
+      <c r="AF38" t="n">
+        <v>-417940</v>
+      </c>
+      <c r="AG38" t="inlineStr">
+        <is>
+          <t>&gt;100</t>
+        </is>
+      </c>
+      <c r="AH38" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="AI38" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="AJ38" t="n">
+        <v>317031.22</v>
+      </c>
+      <c r="AK38" t="n">
+        <v>145228.09</v>
+      </c>
+      <c r="AL38" t="n">
+        <v>-36364.44</v>
+      </c>
+      <c r="AM38" t="n">
+        <v>-446441.38</v>
+      </c>
+      <c r="AN38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO38" t="inlineStr">
+        <is>
+          <t>OD_DA_500kWh_FCROLLING_MEAN_PFLP_LFCNN_LSTM_DAM05.xlsx</t>
+        </is>
+      </c>
+      <c r="AP38" t="n">
+        <v>-80560.36</v>
+      </c>
+      <c r="AQ38" t="n">
+        <v>-189277.37</v>
+      </c>
+      <c r="AR38" t="n">
+        <v>-49477.48</v>
+      </c>
+      <c r="AS38" t="n">
+        <v>-120155.29</v>
+      </c>
+      <c r="AT38" t="inlineStr">
+        <is>
+          <t>MAPE_05</t>
+        </is>
+      </c>
+      <c r="AU38" t="inlineStr">
+        <is>
+          <t>OPTIMISATION_DISPATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-05-15 15:59</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ROLLING_MEAN</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>LP_OPTIMISED</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="F39" t="b">
+        <v>1</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>HYDRO_COUPLED</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>6000</v>
+      </c>
+      <c r="I39" t="n">
+        <v>1</v>
+      </c>
+      <c r="J39" t="n">
+        <v>80</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L39" t="n">
+        <v>15</v>
+      </c>
+      <c r="M39" t="n">
+        <v>5</v>
+      </c>
+      <c r="N39" t="n">
+        <v>8</v>
+      </c>
+      <c r="O39" t="n">
+        <v>48000</v>
+      </c>
+      <c r="P39" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>-269837.73</v>
+      </c>
+      <c r="R39" t="n">
+        <v>1489.65</v>
+      </c>
+      <c r="S39" t="n">
+        <v>-219783</v>
+      </c>
+      <c r="T39" t="n">
+        <v>95488.92</v>
+      </c>
+      <c r="U39" t="n">
+        <v>266</v>
+      </c>
+      <c r="V39" t="n">
+        <v>100</v>
+      </c>
+      <c r="W39" t="n">
+        <v>17190.5</v>
+      </c>
+      <c r="X39" t="n">
+        <v>398.5</v>
+      </c>
+      <c r="Y39" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="Z39" t="n">
+        <v>-30622.68</v>
+      </c>
+      <c r="AA39" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="AB39" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="AC39" t="n">
+        <v>366</v>
+      </c>
+      <c r="AD39" t="n">
+        <v>41698.91</v>
+      </c>
+      <c r="AE39" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="AF39" t="n">
+        <v>-1864737</v>
+      </c>
+      <c r="AG39" t="inlineStr">
+        <is>
+          <t>&gt;100</t>
+        </is>
+      </c>
+      <c r="AH39" t="n">
+        <v>0.705</v>
+      </c>
+      <c r="AI39" t="n">
+        <v>97.8</v>
+      </c>
+      <c r="AJ39" t="n">
+        <v>60544.44</v>
+      </c>
+      <c r="AK39" t="n">
+        <v>145228.09</v>
+      </c>
+      <c r="AL39" t="n">
+        <v>72435.83</v>
+      </c>
+      <c r="AM39" t="n">
+        <v>-309460.47</v>
+      </c>
+      <c r="AN39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO39" t="inlineStr">
+        <is>
+          <t>OD_ID_6000kWh_FCROLLING_MEAN_PFLP_LFCNN_LSTM_DAM05.xlsx</t>
+        </is>
+      </c>
+      <c r="AP39" t="n">
+        <v>-80560.36</v>
+      </c>
+      <c r="AQ39" t="n">
+        <v>-189277.37</v>
+      </c>
+      <c r="AR39" t="n">
+        <v>-50148.62</v>
+      </c>
+      <c r="AS39" t="n">
+        <v>-169634.38</v>
+      </c>
+      <c r="AT39" t="inlineStr">
+        <is>
+          <t>MAPE_05</t>
+        </is>
+      </c>
+      <c r="AU39" t="inlineStr">
+        <is>
+          <t>OPTIMISATION_DISPATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:36</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ROLLING_MEAN</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>LP_OPTIMISED</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="F40" t="b">
+        <v>1</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>HYDRO_COUPLED</t>
+        </is>
+      </c>
+      <c r="H40" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I40" t="n">
+        <v>1</v>
+      </c>
+      <c r="J40" t="n">
+        <v>80</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L40" t="n">
+        <v>15</v>
+      </c>
+      <c r="M40" t="n">
+        <v>5</v>
+      </c>
+      <c r="N40" t="n">
+        <v>8</v>
+      </c>
+      <c r="O40" t="n">
+        <v>24000</v>
+      </c>
+      <c r="P40" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>-269837.73</v>
+      </c>
+      <c r="R40" t="n">
+        <v>4106.21</v>
+      </c>
+      <c r="S40" t="n">
+        <v>-185862.63</v>
+      </c>
+      <c r="T40" t="n">
+        <v>132025.86</v>
+      </c>
+      <c r="U40" t="n">
+        <v>288</v>
+      </c>
+      <c r="V40" t="n">
+        <v>78</v>
+      </c>
+      <c r="W40" t="n">
+        <v>17190.6</v>
+      </c>
+      <c r="X40" t="n">
+        <v>398.5</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="Z40" t="n">
+        <v>-8132.06</v>
+      </c>
+      <c r="AA40" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="AB40" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="AC40" t="n">
+        <v>366</v>
+      </c>
+      <c r="AD40" t="n">
+        <v>54025.26</v>
+      </c>
+      <c r="AE40" t="n">
+        <v>900000</v>
+      </c>
+      <c r="AF40" t="n">
+        <v>-590947</v>
+      </c>
+      <c r="AG40" t="n">
+        <v>30</v>
+      </c>
+      <c r="AH40" t="n">
+        <v>0.859</v>
+      </c>
+      <c r="AI40" t="n">
+        <v>98.2</v>
+      </c>
+      <c r="AJ40" t="n">
+        <v>68280.55</v>
+      </c>
+      <c r="AK40" t="n">
+        <v>145228.09</v>
+      </c>
+      <c r="AL40" t="n">
+        <v>62305.34</v>
+      </c>
+      <c r="AM40" t="n">
+        <v>-258169.03</v>
+      </c>
+      <c r="AN40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO40" t="inlineStr">
+        <is>
+          <t>OD_ID_3000kWh_FCROLLING_MEAN_PFLP_LFCNN_LSTM_DAM05.xlsx</t>
+        </is>
+      </c>
+      <c r="AP40" t="n">
+        <v>-80560.36</v>
+      </c>
+      <c r="AQ40" t="n">
+        <v>-189277.37</v>
+      </c>
+      <c r="AR40" t="n">
+        <v>-49484.64</v>
+      </c>
+      <c r="AS40" t="n">
+        <v>-136377.99</v>
+      </c>
+      <c r="AT40" t="inlineStr">
+        <is>
+          <t>MAPE_05</t>
+        </is>
+      </c>
+      <c r="AU40" t="inlineStr">
+        <is>
+          <t>OPTIMISATION_DISPATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-05-15 17:02</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ROLLING_MEAN</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>LP_OPTIMISED</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="F41" t="b">
+        <v>1</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>HYDRO_COUPLED</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I41" t="n">
+        <v>1</v>
+      </c>
+      <c r="J41" t="n">
+        <v>80</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L41" t="n">
+        <v>15</v>
+      </c>
+      <c r="M41" t="n">
+        <v>5</v>
+      </c>
+      <c r="N41" t="n">
+        <v>8</v>
+      </c>
+      <c r="O41" t="n">
+        <v>8000</v>
+      </c>
+      <c r="P41" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>-269837.73</v>
+      </c>
+      <c r="R41" t="n">
+        <v>6083.47</v>
+      </c>
+      <c r="S41" t="n">
+        <v>-171028.44</v>
+      </c>
+      <c r="T41" t="n">
+        <v>148837.3</v>
+      </c>
+      <c r="U41" t="n">
+        <v>299</v>
+      </c>
+      <c r="V41" t="n">
+        <v>67</v>
+      </c>
+      <c r="W41" t="n">
+        <v>17190.6</v>
+      </c>
+      <c r="X41" t="n">
+        <v>398.5</v>
+      </c>
+      <c r="Y41" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="Z41" t="n">
+        <v>-73.42</v>
+      </c>
+      <c r="AA41" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="AB41" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="AC41" t="n">
+        <v>366</v>
+      </c>
+      <c r="AD41" t="n">
+        <v>45274.79</v>
+      </c>
+      <c r="AE41" t="n">
+        <v>300000</v>
+      </c>
+      <c r="AF41" t="n">
+        <v>83248</v>
+      </c>
+      <c r="AG41" t="n">
+        <v>8</v>
+      </c>
+      <c r="AH41" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="AI41" t="n">
+        <v>98</v>
+      </c>
+      <c r="AJ41" t="n">
+        <v>73665.88</v>
+      </c>
+      <c r="AK41" t="n">
+        <v>145228.09</v>
+      </c>
+      <c r="AL41" t="n">
+        <v>45472.25</v>
+      </c>
+      <c r="AM41" t="n">
+        <v>-238684.27</v>
+      </c>
+      <c r="AN41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO41" t="inlineStr">
+        <is>
+          <t>OD_ID_1000kWh_FCROLLING_MEAN_PFLP_LFCNN_LSTM_DAM05.xlsx</t>
+        </is>
+      </c>
+      <c r="AP41" t="n">
+        <v>-80560.36</v>
+      </c>
+      <c r="AQ41" t="n">
+        <v>-189277.37</v>
+      </c>
+      <c r="AR41" t="n">
+        <v>-49456.76</v>
+      </c>
+      <c r="AS41" t="n">
+        <v>-121571.68</v>
+      </c>
+      <c r="AT41" t="inlineStr">
+        <is>
+          <t>MAPE_05</t>
+        </is>
+      </c>
+      <c r="AU41" t="inlineStr">
+        <is>
+          <t>OPTIMISATION_DISPATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-05-15 17:17</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ROLLING_MEAN</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>LP_OPTIMISED</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="F42" t="b">
+        <v>1</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>HYDRO_COUPLED</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>200</v>
+      </c>
+      <c r="I42" t="n">
+        <v>1</v>
+      </c>
+      <c r="J42" t="n">
+        <v>80</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L42" t="n">
+        <v>15</v>
+      </c>
+      <c r="M42" t="n">
+        <v>5</v>
+      </c>
+      <c r="N42" t="n">
+        <v>8</v>
+      </c>
+      <c r="O42" t="n">
+        <v>1600</v>
+      </c>
+      <c r="P42" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>-269837.73</v>
+      </c>
+      <c r="R42" t="n">
+        <v>7374.94</v>
+      </c>
+      <c r="S42" t="n">
+        <v>-166298.96</v>
+      </c>
+      <c r="T42" t="n">
+        <v>154858.26</v>
+      </c>
+      <c r="U42" t="n">
+        <v>305</v>
+      </c>
+      <c r="V42" t="n">
+        <v>61</v>
+      </c>
+      <c r="W42" t="n">
+        <v>17188.8</v>
+      </c>
+      <c r="X42" t="n">
+        <v>401.2</v>
+      </c>
+      <c r="Y42" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="Z42" t="n">
+        <v>1483.97</v>
+      </c>
+      <c r="AA42" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="AB42" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="AC42" t="n">
+        <v>366</v>
+      </c>
+      <c r="AD42" t="n">
+        <v>21123.83</v>
+      </c>
+      <c r="AE42" t="n">
+        <v>60000</v>
+      </c>
+      <c r="AF42" t="n">
+        <v>138721</v>
+      </c>
+      <c r="AG42" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="AH42" t="n">
+        <v>0.374</v>
+      </c>
+      <c r="AI42" t="n">
+        <v>95.90000000000001</v>
+      </c>
+      <c r="AJ42" t="n">
+        <v>77122.12</v>
+      </c>
+      <c r="AK42" t="n">
+        <v>145228.09</v>
+      </c>
+      <c r="AL42" t="n">
+        <v>19697.74</v>
+      </c>
+      <c r="AM42" t="n">
+        <v>-234562.17</v>
+      </c>
+      <c r="AN42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO42" t="inlineStr">
+        <is>
+          <t>OD_ID_200kWh_FCROLLING_MEAN_PFLP_LFCNN_LSTM_DAM05.xlsx</t>
+        </is>
+      </c>
+      <c r="AP42" t="n">
+        <v>-80560.36</v>
+      </c>
+      <c r="AQ42" t="n">
+        <v>-189277.37</v>
+      </c>
+      <c r="AR42" t="n">
+        <v>-49650.32</v>
+      </c>
+      <c r="AS42" t="n">
+        <v>-116648.64</v>
+      </c>
+      <c r="AT42" t="inlineStr">
+        <is>
+          <t>MAPE_05</t>
+        </is>
+      </c>
+      <c r="AU42" t="inlineStr">
+        <is>
+          <t>OPTIMISATION_DISPATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-05-16 12:17</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ROLLING_MEAN</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>LP_OPTIMISED</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="F43" t="b">
+        <v>1</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>HYDRO_COUPLED</t>
+        </is>
+      </c>
+      <c r="H43" t="n">
+        <v>200</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J43" t="n">
+        <v>80</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L43" t="n">
+        <v>15</v>
+      </c>
+      <c r="M43" t="n">
+        <v>5</v>
+      </c>
+      <c r="N43" t="n">
+        <v>8</v>
+      </c>
+      <c r="O43" t="n">
+        <v>1600</v>
+      </c>
+      <c r="P43" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>-269837.73</v>
+      </c>
+      <c r="R43" t="n">
+        <v>7360.47</v>
+      </c>
+      <c r="S43" t="n">
+        <v>-165979.81</v>
+      </c>
+      <c r="T43" t="n">
+        <v>155162.93</v>
+      </c>
+      <c r="U43" t="n">
+        <v>306</v>
+      </c>
+      <c r="V43" t="n">
+        <v>60</v>
+      </c>
+      <c r="W43" t="n">
+        <v>17188.8</v>
+      </c>
+      <c r="X43" t="n">
+        <v>401</v>
+      </c>
+      <c r="Y43" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="Z43" t="n">
+        <v>1503.04</v>
+      </c>
+      <c r="AA43" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="AB43" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="AC43" t="n">
+        <v>366</v>
+      </c>
+      <c r="AD43" t="n">
+        <v>12533.24</v>
+      </c>
+      <c r="AE43" t="n">
+        <v>60000</v>
+      </c>
+      <c r="AF43" t="n">
+        <v>51426</v>
+      </c>
+      <c r="AG43" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="AH43" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AI43" t="n">
+        <v>96.2</v>
+      </c>
+      <c r="AJ43" t="n">
+        <v>77607.92999999999</v>
+      </c>
+      <c r="AK43" t="n">
+        <v>145228.09</v>
+      </c>
+      <c r="AL43" t="n">
+        <v>11064.54</v>
+      </c>
+      <c r="AM43" t="n">
+        <v>-234724.23</v>
+      </c>
+      <c r="AN43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO43" t="inlineStr">
+        <is>
+          <t>OD_ID_200kWh_FCROLLING_MEAN_PFLP_LFCNN_LSTM_DAM05.xlsx</t>
+        </is>
+      </c>
+      <c r="AP43" t="n">
+        <v>-80560.36</v>
+      </c>
+      <c r="AQ43" t="n">
+        <v>-189277.37</v>
+      </c>
+      <c r="AR43" t="n">
+        <v>-50017.15</v>
+      </c>
+      <c r="AS43" t="n">
+        <v>-115962.66</v>
+      </c>
+      <c r="AT43" t="inlineStr">
+        <is>
+          <t>MAPE_05</t>
+        </is>
+      </c>
+      <c r="AU43" t="inlineStr">
+        <is>
+          <t>OPTIMISATION_DISPATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-05-16 12:34</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ROLLING_MEAN</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>LP_OPTIMISED</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="F44" t="b">
+        <v>1</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>HYDRO_COUPLED</t>
+        </is>
+      </c>
+      <c r="H44" t="n">
+        <v>500</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J44" t="n">
+        <v>80</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L44" t="n">
+        <v>15</v>
+      </c>
+      <c r="M44" t="n">
+        <v>5</v>
+      </c>
+      <c r="N44" t="n">
+        <v>8</v>
+      </c>
+      <c r="O44" t="n">
+        <v>4000</v>
+      </c>
+      <c r="P44" t="n">
+        <v>-43944.54</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>-269837.73</v>
+      </c>
+      <c r="R44" t="n">
+        <v>7035.59</v>
+      </c>
+      <c r="S44" t="n">
+        <v>-167087.54</v>
+      </c>
+      <c r="T44" t="n">
+        <v>153730.32</v>
+      </c>
+      <c r="U44" t="n">
+        <v>302</v>
+      </c>
+      <c r="V44" t="n">
+        <v>64</v>
+      </c>
+      <c r="W44" t="n">
+        <v>17189.8</v>
+      </c>
+      <c r="X44" t="n">
+        <v>399.7</v>
+      </c>
+      <c r="Y44" t="n">
+        <v>24</v>
+      </c>
+      <c r="Z44" t="n">
+        <v>1359.24</v>
+      </c>
+      <c r="AA44" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="AB44" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="AC44" t="n">
+        <v>366</v>
+      </c>
+      <c r="AD44" t="n">
+        <v>24333.06</v>
+      </c>
+      <c r="AE44" t="n">
+        <v>150000</v>
+      </c>
+      <c r="AF44" t="n">
+        <v>58625</v>
+      </c>
+      <c r="AG44" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="AH44" t="n">
+        <v>0.626</v>
+      </c>
+      <c r="AI44" t="n">
+        <v>97.59999999999999</v>
+      </c>
+      <c r="AJ44" t="n">
+        <v>75910.10000000001</v>
+      </c>
+      <c r="AK44" t="n">
+        <v>145228.09</v>
+      </c>
+      <c r="AL44" t="n">
+        <v>23040.49</v>
+      </c>
+      <c r="AM44" t="n">
+        <v>-234602.81</v>
+      </c>
+      <c r="AN44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO44" t="inlineStr">
+        <is>
+          <t>OD_ID_500kWh_FCROLLING_MEAN_PFLP_LFCNN_LSTM_DAM05.xlsx</t>
+        </is>
+      </c>
+      <c r="AP44" t="n">
+        <v>-80560.36</v>
+      </c>
+      <c r="AQ44" t="n">
+        <v>-189277.37</v>
+      </c>
+      <c r="AR44" t="n">
+        <v>-49567.9</v>
+      </c>
+      <c r="AS44" t="n">
+        <v>-117519.64</v>
+      </c>
+      <c r="AT44" t="inlineStr">
+        <is>
+          <t>MAPE_05</t>
+        </is>
+      </c>
+      <c r="AU44" t="inlineStr">
+        <is>
+          <t>OPTIMISATION_DISPATCH</t>
         </is>
       </c>
     </row>

</xml_diff>